<commit_message>
Make the sensitivity tables live formulas instead of hardcoded values
The DCF discount-rate sensitivity grid and Reverse Test Route 1 held
values computed outside the workbook and written in as literals, so
they would not respond to a change in any assumption. Both now compute
in the sheet, reading the free cash flow rows from the Projections tab
and the terminal growth rate and net debt from their source cells:

  =NPV(rate, FCF C:H)
   + (FCF_FY32 * (1 + g) / (rate - g)) / (1 + rate)^6
   - net debt

Route 2's enterprise value for the Moderate case is likewise derived
rather than pasted. Values are unchanged; they are now reproducible
from the workbook itself, which matters when the client's accountant
tests the model.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ps4mzHm443DfwaJ7XP6HFW
</commit_message>
<xml_diff>
--- a/03-valuation/Valuation_Model_Astral_School.xlsx
+++ b/03-valuation/Valuation_Model_Astral_School.xlsx
@@ -5001,13 +5001,16 @@
       <c r="B55" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="C55" s="10" t="n">
+      <c r="C55" s="10">
+        <f>(NPV($B55,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B55-Assumptions!$C$10))/(1+$B55)^6-'Audited Base'!$C$37)/100000</f>
         <v>374.3478715007848</v>
       </c>
-      <c r="D55" s="10" t="n">
+      <c r="D55" s="10">
+        <f>(NPV($B55,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B55-Assumptions!$C$10))/(1+$B55)^6-'Audited Base'!$C$37)/100000</f>
         <v>681.4881821843841</v>
       </c>
-      <c r="E55" s="10" t="n">
+      <c r="E55" s="10">
+        <f>(NPV($B55,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B55-Assumptions!$C$10))/(1+$B55)^6-'Audited Base'!$C$37)/100000</f>
         <v>965.800285823213</v>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -5020,13 +5023,16 @@
       <c r="B56" s="41" t="n">
         <v>0.14</v>
       </c>
-      <c r="C56" s="10" t="n">
+      <c r="C56" s="10">
+        <f>(NPV($B56,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B56-Assumptions!$C$10))/(1+$B56)^6-'Audited Base'!$C$37)/100000</f>
         <v>133.8565576063081</v>
       </c>
-      <c r="D56" s="10" t="n">
+      <c r="D56" s="10">
+        <f>(NPV($B56,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B56-Assumptions!$C$10))/(1+$B56)^6-'Audited Base'!$C$37)/100000</f>
         <v>288.1115833915733</v>
       </c>
-      <c r="E56" s="10" t="n">
+      <c r="E56" s="10">
+        <f>(NPV($B56,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B56-Assumptions!$C$10))/(1+$B56)^6-'Audited Base'!$C$37)/100000</f>
         <v>431.7502768148422</v>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
@@ -5035,13 +5041,16 @@
       <c r="B57" s="41" t="n">
         <v>0.16</v>
       </c>
-      <c r="C57" s="10" t="n">
+      <c r="C57" s="10">
+        <f>(NPV($B57,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B57-Assumptions!$C$10))/(1+$B57)^6-'Audited Base'!$C$37)/100000</f>
         <v>79.79707725209288</v>
       </c>
-      <c r="D57" s="10" t="n">
+      <c r="D57" s="10">
+        <f>(NPV($B57,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B57-Assumptions!$C$10))/(1+$B57)^6-'Audited Base'!$C$37)/100000</f>
         <v>200.096640803215</v>
       </c>
-      <c r="E57" s="10" t="n">
+      <c r="E57" s="10">
+        <f>(NPV($B57,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B57-Assumptions!$C$10))/(1+$B57)^6-'Audited Base'!$C$37)/100000</f>
         <v>312.3823670974401</v>
       </c>
       <c r="F57" s="7" t="inlineStr"/>
@@ -5050,14 +5059,17 @@
       <c r="B58" s="41" t="n">
         <v>0.19</v>
       </c>
-      <c r="C58" s="13" t="n">
-        <v>28.16905374859341</v>
-      </c>
-      <c r="D58" s="13" t="n">
-        <v>116.3892066847429</v>
-      </c>
-      <c r="E58" s="13" t="n">
-        <v>198.967253988027</v>
+      <c r="C58" s="13">
+        <f>(NPV($B58,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B58-Assumptions!$C$10))/(1+$B58)^6-'Audited Base'!$C$37)/100000</f>
+        <v>28.169053748593406</v>
+      </c>
+      <c r="D58" s="13">
+        <f>(NPV($B58,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B58-Assumptions!$C$10))/(1+$B58)^6-'Audited Base'!$C$37)/100000</f>
+        <v>116.38920668474287</v>
+      </c>
+      <c r="E58" s="13">
+        <f>(NPV($B58,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B58-Assumptions!$C$10))/(1+$B58)^6-'Audited Base'!$C$37)/100000</f>
+        <v>198.96725398802698</v>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
@@ -5069,14 +5081,17 @@
       <c r="B59" s="41" t="n">
         <v>0.22</v>
       </c>
-      <c r="C59" s="10" t="n">
+      <c r="C59" s="10">
+        <f>(NPV($B59,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B59-Assumptions!$C$10))/(1+$B59)^6-'Audited Base'!$C$37)/100000</f>
         <v>-4.805191819553096</v>
       </c>
-      <c r="D59" s="10" t="n">
-        <v>63.23037248332314</v>
-      </c>
-      <c r="E59" s="10" t="n">
-        <v>127.0448723839584</v>
+      <c r="D59" s="10">
+        <f>(NPV($B59,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B59-Assumptions!$C$10))/(1+$B59)^6-'Audited Base'!$C$37)/100000</f>
+        <v>63.230372483323144</v>
+      </c>
+      <c r="E59" s="10">
+        <f>(NPV($B59,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B59-Assumptions!$C$10))/(1+$B59)^6-'Audited Base'!$C$37)/100000</f>
+        <v>127.04487238395843</v>
       </c>
       <c r="F59" s="7" t="inlineStr"/>
     </row>
@@ -5084,13 +5099,16 @@
       <c r="B60" s="41" t="n">
         <v>0.25</v>
       </c>
-      <c r="C60" s="10" t="n">
-        <v>-27.57068399112443</v>
-      </c>
-      <c r="D60" s="10" t="n">
+      <c r="C60" s="10">
+        <f>(NPV($B60,Projections!$C$22:$H$22)+(Projections!$H$22*(1+Assumptions!$C$10)/($B60-Assumptions!$C$10))/(1+$B60)^6-'Audited Base'!$C$37)/100000</f>
+        <v>-27.570683991124426</v>
+      </c>
+      <c r="D60" s="10">
+        <f>(NPV($B60,Projections!$C$41:$H$41)+(Projections!$H$41*(1+Assumptions!$C$10)/($B60-Assumptions!$C$10))/(1+$B60)^6-'Audited Base'!$C$37)/100000</f>
         <v>26.75524477289753</v>
       </c>
-      <c r="E60" s="10" t="n">
+      <c r="E60" s="10">
+        <f>(NPV($B60,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B60-Assumptions!$C$10))/(1+$B60)^6-'Audited Base'!$C$37)/100000</f>
         <v>77.7760336626985</v>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
@@ -5602,7 +5620,8 @@
       <c r="B12" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="8">
+        <f>NPV($B12,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B12-Assumptions!$C$10))/(1+$B12)^6-'Audited Base'!$C$37</f>
         <v>96580028.5823213</v>
       </c>
       <c r="D12" s="20">
@@ -5619,7 +5638,8 @@
       <c r="B13" s="41" t="n">
         <v>0.11</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="8">
+        <f>NPV($B13,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B13-Assumptions!$C$10))/(1+$B13)^6-'Audited Base'!$C$37</f>
         <v>76452909.02366123</v>
       </c>
       <c r="D13" s="18">
@@ -5632,8 +5652,9 @@
       <c r="B14" s="41" t="n">
         <v>0.12</v>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>62135683.84624141</v>
+      <c r="C14" s="8">
+        <f>NPV($B14,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B14-Assumptions!$C$10))/(1+$B14)^6-'Audited Base'!$C$37</f>
+        <v>62135683.846241415</v>
       </c>
       <c r="D14" s="18">
         <f>C14/$C$6</f>
@@ -5645,7 +5666,8 @@
       <c r="B15" s="41" t="n">
         <v>0.14</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="8">
+        <f>NPV($B15,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B15-Assumptions!$C$10))/(1+$B15)^6-'Audited Base'!$C$37</f>
         <v>43175027.68148422</v>
       </c>
       <c r="D15" s="18">
@@ -5658,8 +5680,9 @@
       <c r="B16" s="41" t="n">
         <v>0.19</v>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>19896725.3988027</v>
+      <c r="C16" s="8">
+        <f>NPV($B16,Projections!$C$60:$H$60)+(Projections!$H$60*(1+Assumptions!$C$10)/($B16-Assumptions!$C$10))/(1+$B16)^6-'Audited Base'!$C$37</f>
+        <v>19896725.398802698</v>
       </c>
       <c r="D16" s="18">
         <f>C16/$C$6</f>

</xml_diff>